<commit_message>
fixed alternate names and added sp6,sp4 and current forestgeo column
</commit_message>
<xml_diff>
--- a/tocheck/plotsbci_not_garwood.xlsx
+++ b/tocheck/plotsbci_not_garwood.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AY13"/>
+  <dimension ref="A1:AY7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -739,7 +739,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>Jupunba idiopoda</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
@@ -821,16 +821,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ardiba</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Ardisia bartlettii</t>
+          <t>buchca</t>
         </is>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -842,41 +837,46 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>bci50ha</t>
+          <t>bcimultiplots</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Ericales</t>
+          <t>Myrtales</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Primulaceae</t>
+          <t>Combretaceae</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Ardisia</t>
+          <t>Terminalia</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>bartletii</t>
+          <t>tetraphylla</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Lundell</t>
+          <t>(Aubl.) Gere &amp; Boatwr.</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Buchenavia tetraphylla, Buchenavia capitata</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>R. Pérez 2125 (PMA, SCZ)</t>
+          <t>S. Aguilar 951 (PMA, SCZ)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -886,12 +886,12 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Ardisia bartletii</t>
+          <t>Terminalia tetraphylla</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Ardisia bartletii</t>
+          <t>Terminalia tetraphylla</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -901,12 +901,12 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Ardisia bartletii</t>
+          <t>Terminalia tetraphylla</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Lundell</t>
+          <t>(Aubl.) Gere &amp; Boatwr.</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -921,12 +921,12 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>2647592</t>
+          <t>3016509</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>18048-2</t>
+          <t>77164595-1</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
@@ -936,47 +936,47 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>2647592</t>
+          <t>3016509</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>18048-2</t>
+          <t>77164595-1</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>18048-2</t>
+          <t>77164595-1</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>Terminalia tetraphylla</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>Ardisia bartletii</t>
+          <t>Terminalia tetraphylla</t>
         </is>
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>Lundell</t>
+          <t>(Aubl.) Gere &amp; Boatwr.</t>
         </is>
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>Primulaceae</t>
+          <t>Combretaceae</t>
         </is>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>Ardisia</t>
+          <t>Terminalia</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>bartletii</t>
+          <t>tetraphylla</t>
         </is>
       </c>
       <c r="AN3" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="AO3" t="inlineStr">
         <is>
-          <t>shrub or tree</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="AP3" t="inlineStr">
@@ -996,17 +996,17 @@
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
-          <t>Ardisia bartletii</t>
+          <t>Terminalia tetraphylla</t>
         </is>
       </c>
       <c r="AR3" t="inlineStr">
         <is>
-          <t>Lundell</t>
+          <t>(Aubl.) Gere &amp; Boatwr.</t>
         </is>
       </c>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>Primulaceae</t>
+          <t>Combretaceae</t>
         </is>
       </c>
       <c r="AT3" t="inlineStr">
@@ -1021,28 +1021,23 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>Ardisia</t>
+          <t>Terminalia</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>bartletii</t>
-        </is>
-      </c>
-      <c r="AY3" t="inlineStr">
-        <is>
-          <t>ARDB</t>
+          <t>tetraphylla</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>buchca</t>
+          <t>cupasc</t>
         </is>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -1054,46 +1049,41 @@
         <v>0</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>bcimultiplots</t>
+          <t>bci50ha</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Myrtales</t>
+          <t>Sapindales</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Combretaceae</t>
+          <t>Sapindaceae</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Terminalia</t>
+          <t>Cupania</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>tetraphylla</t>
+          <t>scrobiculata</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>(Aubl.) Gere &amp; Boatwr.</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Buchenavia tetraphylla, Buchenavia capitata</t>
+          <t>Rich.</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>S. Aguilar 951 (PMA, SCZ)</t>
+          <t>R. Pérez 2474 (PMA, SCZ)</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -1103,12 +1093,12 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Terminalia tetraphylla</t>
+          <t>Cupania scrobiculata</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Terminalia tetraphylla</t>
+          <t>Cupania scrobiculata</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -1118,12 +1108,12 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Terminalia tetraphylla</t>
+          <t>Cupania scrobiculata</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>(Aubl.) Gere &amp; Boatwr.</t>
+          <t>Rich.</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -1138,12 +1128,12 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>3016509</t>
+          <t>2747671</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>77164595-1</t>
+          <t>782556-1</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -1153,47 +1143,47 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>3016509</t>
+          <t>2747671</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>77164595-1</t>
+          <t>782556-1</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>77164595-1</t>
+          <t>782556-1</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>Cupania scrobiculata</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>Terminalia tetraphylla</t>
+          <t>Cupania scrobiculata</t>
         </is>
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>(Aubl.) Gere &amp; Boatwr.</t>
+          <t>Rich.</t>
         </is>
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>Combretaceae</t>
+          <t>Sapindaceae</t>
         </is>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>Terminalia</t>
+          <t>Cupania</t>
         </is>
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>tetraphylla</t>
+          <t>scrobiculata</t>
         </is>
       </c>
       <c r="AN4" t="inlineStr">
@@ -1203,7 +1193,7 @@
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>shrub or tree</t>
         </is>
       </c>
       <c r="AP4" t="inlineStr">
@@ -1213,17 +1203,17 @@
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
-          <t>Terminalia tetraphylla</t>
+          <t>Cupania scrobiculata</t>
         </is>
       </c>
       <c r="AR4" t="inlineStr">
         <is>
-          <t>(Aubl.) Gere &amp; Boatwr.</t>
+          <t>Rich.</t>
         </is>
       </c>
       <c r="AS4" t="inlineStr">
         <is>
-          <t>Combretaceae</t>
+          <t>Sapindaceae</t>
         </is>
       </c>
       <c r="AT4" t="inlineStr">
@@ -1238,69 +1228,74 @@
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>Terminalia</t>
+          <t>Cupania</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>tetraphylla</t>
+          <t>scrobiculata</t>
+        </is>
+      </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>CUP2</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>cupasc</t>
+          <t>myr2fl</t>
         </is>
       </c>
       <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
         <v>1</v>
       </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>bci50ha</t>
+          <t>bcimultiplots</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Sapindales</t>
+          <t>Myrtales</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Sapindaceae</t>
+          <t>Myrtaceae</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Cupania</t>
+          <t>Myrciaria</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>scrobiculata</t>
+          <t>floribunda</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Rich.</t>
+          <t>(H. West ex Willd.) O. Berg</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>R. Pérez 2474 (PMA, SCZ)</t>
+          <t>R. Pérez 2347 (PMA, SCZ)</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -1310,12 +1305,12 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Cupania scrobiculata</t>
+          <t>Myrciaria floribunda</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Cupania scrobiculata</t>
+          <t>Myrciaria floribunda</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -1325,12 +1320,12 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Cupania scrobiculata</t>
+          <t>Myrciaria floribunda</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>Rich.</t>
+          <t>(H.West ex Willd.) O.Berg</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
@@ -1345,12 +1340,12 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>2747671</t>
+          <t>131815</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>782556-1</t>
+          <t>599327-1</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -1360,47 +1355,47 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>2747671</t>
+          <t>131815</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>782556-1</t>
+          <t>599327-1</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>782556-1</t>
+          <t>599327-1</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>Myrciaria floribunda</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>Cupania scrobiculata</t>
+          <t>Myrciaria floribunda</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>Rich.</t>
+          <t>(H.West ex Willd.) O.Berg</t>
         </is>
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>Sapindaceae</t>
+          <t>Myrtaceae</t>
         </is>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>Cupania</t>
+          <t>Myrciaria</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>scrobiculata</t>
+          <t>floribunda</t>
         </is>
       </c>
       <c r="AN5" t="inlineStr">
@@ -1420,17 +1415,17 @@
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>Cupania scrobiculata</t>
+          <t>Myrciaria floribunda</t>
         </is>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>Rich.</t>
+          <t>(H.West ex Willd.) O.Berg</t>
         </is>
       </c>
       <c r="AS5" t="inlineStr">
         <is>
-          <t>Sapindaceae</t>
+          <t>Myrtaceae</t>
         </is>
       </c>
       <c r="AT5" t="inlineStr">
@@ -1445,24 +1440,24 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>Cupania</t>
+          <t>Myrciaria</t>
         </is>
       </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>scrobiculata</t>
+          <t>floribunda</t>
         </is>
       </c>
       <c r="AY5" t="inlineStr">
         <is>
-          <t>CUP2</t>
+          <t>MYRF</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>mataap</t>
+          <t>nectcu</t>
         </is>
       </c>
       <c r="C6">
@@ -1478,7 +1473,7 @@
         <v>0</v>
       </c>
       <c r="G6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -1487,37 +1482,32 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Sapindales</t>
+          <t>Laurales</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Sapindaceae</t>
+          <t>Lauraceae</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Matayba</t>
+          <t>Nectandra</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>oppositifolia</t>
+          <t>cuspidata</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Britton</t>
+          <t>Nees &amp; Mart.</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Matayba apetala</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>R. Pérez 2416 (PMA, SCZ)</t>
+          <t>Nectandra gentlei</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1527,12 +1517,12 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Matayba oppositifolia</t>
+          <t>Nectandra cuspidata</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Matayba oppositifolia</t>
+          <t>Nectandra cuspidata</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1542,12 +1532,12 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Matayba oppositifolia</t>
+          <t>Nectandra cuspidata</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>(A.Rich.) Britton</t>
+          <t>Nees &amp; Mart.</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
@@ -1562,12 +1552,12 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>2510244</t>
+          <t>2379054</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>154460-2</t>
+          <t>281229-2</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -1577,47 +1567,47 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>2510244</t>
+          <t>2379054</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>154460-2</t>
+          <t>281229-2</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>154460-2</t>
+          <t>281229-2</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>Nectandra cuspidata</t>
         </is>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>Matayba oppositifolia</t>
+          <t>Nectandra cuspidata</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>(A.Rich.) Britton</t>
+          <t>Nees &amp; Mart.</t>
         </is>
       </c>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>Sapindaceae</t>
+          <t>Lauraceae</t>
         </is>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>Matayba</t>
+          <t>Nectandra</t>
         </is>
       </c>
       <c r="AK6" t="inlineStr">
         <is>
-          <t>oppositifolia</t>
+          <t>cuspidata</t>
         </is>
       </c>
       <c r="AN6" t="inlineStr">
@@ -1637,17 +1627,17 @@
       </c>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>Matayba oppositifolia</t>
+          <t>Nectandra cuspidata</t>
         </is>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
-          <t>(A.Rich.) Britton</t>
+          <t>Nees &amp; Mart.</t>
         </is>
       </c>
       <c r="AS6" t="inlineStr">
         <is>
-          <t>Sapindaceae</t>
+          <t>Lauraceae</t>
         </is>
       </c>
       <c r="AT6" t="inlineStr">
@@ -1662,24 +1652,24 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>Matayba</t>
+          <t>Nectandra</t>
         </is>
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>oppositifolia</t>
+          <t>cuspidata</t>
         </is>
       </c>
       <c r="AY6" t="inlineStr">
         <is>
-          <t>MATA</t>
+          <t>NEC2</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>myr2fl</t>
+          <t>unonpa</t>
         </is>
       </c>
       <c r="C7">
@@ -1704,32 +1694,32 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Myrtales</t>
+          <t>Magnoliales</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Myrtaceae</t>
+          <t>Annonaceae</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Myrciaria</t>
+          <t>Unonopsis</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>floribunda</t>
+          <t>panamensis</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>(H. West ex Willd.) O. Berg</t>
+          <t>R.E. Fr.</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>R. Pérez 2347 (PMA, SCZ)</t>
+          <t>R. Pérez 2303 (PMA, SCZ)</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1739,12 +1729,12 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Myrciaria floribunda</t>
+          <t>Unonopsis panamensis</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Myrciaria floribunda</t>
+          <t>Unonopsis panamensis</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1754,12 +1744,12 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Myrciaria floribunda</t>
+          <t>Unonopsis panamensis</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>(H.West ex Willd.) O.Berg</t>
+          <t>R.E.Fr.</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
@@ -1774,12 +1764,12 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>131815</t>
+          <t>2447472</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>599327-1</t>
+          <t>259517-2</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1789,47 +1779,47 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>131815</t>
+          <t>2447472</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>599327-1</t>
+          <t>259517-2</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>599327-1</t>
+          <t>259517-2</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>Unonopsis panamensis</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>Myrciaria floribunda</t>
+          <t>Unonopsis panamensis</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>(H.West ex Willd.) O.Berg</t>
+          <t>R.E.Fr.</t>
         </is>
       </c>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>Myrtaceae</t>
+          <t>Annonaceae</t>
         </is>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>Myrciaria</t>
+          <t>Unonopsis</t>
         </is>
       </c>
       <c r="AK7" t="inlineStr">
         <is>
-          <t>floribunda</t>
+          <t>panamensis</t>
         </is>
       </c>
       <c r="AN7" t="inlineStr">
@@ -1839,7 +1829,7 @@
       </c>
       <c r="AO7" t="inlineStr">
         <is>
-          <t>shrub or tree</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="AP7" t="inlineStr">
@@ -1849,17 +1839,17 @@
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>Myrciaria floribunda</t>
+          <t>Unonopsis panamensis</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>(H.West ex Willd.) O.Berg</t>
+          <t>R.E.Fr.</t>
         </is>
       </c>
       <c r="AS7" t="inlineStr">
         <is>
-          <t>Myrtaceae</t>
+          <t>Annonaceae</t>
         </is>
       </c>
       <c r="AT7" t="inlineStr">
@@ -1874,1067 +1864,15 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>Myrciaria</t>
+          <t>Unonopsis</t>
         </is>
       </c>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>floribunda</t>
+          <t>panamensis</t>
         </is>
       </c>
       <c r="AY7" t="inlineStr">
-        <is>
-          <t>MYRF</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>myrcze</t>
-        </is>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="G8">
-        <v>1</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>bcimultiplots</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Myrtales</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Myrtaceae</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Myrcia</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>tomentosa</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>(Aubl.) DC.</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Aulomyrcia tomentosa, Aulomyrcia zetekiana</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>Freestanding</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>Myrcia tomentosa</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>Myrcia tomentosa</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>species</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>Myrcia tomentosa</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>(Aubl.) DC.</t>
-        </is>
-      </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>Accepted</t>
-        </is>
-      </c>
-      <c r="Z8" t="inlineStr">
-        <is>
-          <t>131684</t>
-        </is>
-      </c>
-      <c r="AA8" t="inlineStr">
-        <is>
-          <t>599215-1</t>
-        </is>
-      </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t>131684</t>
-        </is>
-      </c>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>599215-1</t>
-        </is>
-      </c>
-      <c r="AE8" t="inlineStr">
-        <is>
-          <t>599215-1</t>
-        </is>
-      </c>
-      <c r="AF8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AG8" t="inlineStr">
-        <is>
-          <t>Myrcia tomentosa</t>
-        </is>
-      </c>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>(Aubl.) DC.</t>
-        </is>
-      </c>
-      <c r="AI8" t="inlineStr">
-        <is>
-          <t>Myrtaceae</t>
-        </is>
-      </c>
-      <c r="AJ8" t="inlineStr">
-        <is>
-          <t>Myrcia</t>
-        </is>
-      </c>
-      <c r="AK8" t="inlineStr">
-        <is>
-          <t>tomentosa</t>
-        </is>
-      </c>
-      <c r="AN8" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="AO8" t="inlineStr">
-        <is>
-          <t>shrub or tree</t>
-        </is>
-      </c>
-      <c r="AP8" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AQ8" t="inlineStr">
-        <is>
-          <t>Myrcia tomentosa</t>
-        </is>
-      </c>
-      <c r="AR8" t="inlineStr">
-        <is>
-          <t>(Aubl.) DC.</t>
-        </is>
-      </c>
-      <c r="AS8" t="inlineStr">
-        <is>
-          <t>Myrtaceae</t>
-        </is>
-      </c>
-      <c r="AT8" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AU8" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AV8" t="inlineStr">
-        <is>
-          <t>Myrcia</t>
-        </is>
-      </c>
-      <c r="AW8" t="inlineStr">
-        <is>
-          <t>tomentosa</t>
-        </is>
-      </c>
-      <c r="AY8" t="inlineStr">
-        <is>
-          <t>MYRZ</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>nectcu</t>
-        </is>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9">
-        <v>1</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>bcimultiplots</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Laurales</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Lauraceae</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Nectandra</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>cuspidata</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Nees &amp; Mart.</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>Nectandra gentlei</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>Freestanding</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>Nectandra cuspidata</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>Nectandra cuspidata</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>species</t>
-        </is>
-      </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>Nectandra cuspidata</t>
-        </is>
-      </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>Nees &amp; Mart.</t>
-        </is>
-      </c>
-      <c r="X9" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>Accepted</t>
-        </is>
-      </c>
-      <c r="Z9" t="inlineStr">
-        <is>
-          <t>2379054</t>
-        </is>
-      </c>
-      <c r="AA9" t="inlineStr">
-        <is>
-          <t>281229-2</t>
-        </is>
-      </c>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>2379054</t>
-        </is>
-      </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t>281229-2</t>
-        </is>
-      </c>
-      <c r="AE9" t="inlineStr">
-        <is>
-          <t>281229-2</t>
-        </is>
-      </c>
-      <c r="AF9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AG9" t="inlineStr">
-        <is>
-          <t>Nectandra cuspidata</t>
-        </is>
-      </c>
-      <c r="AH9" t="inlineStr">
-        <is>
-          <t>Nees &amp; Mart.</t>
-        </is>
-      </c>
-      <c r="AI9" t="inlineStr">
-        <is>
-          <t>Lauraceae</t>
-        </is>
-      </c>
-      <c r="AJ9" t="inlineStr">
-        <is>
-          <t>Nectandra</t>
-        </is>
-      </c>
-      <c r="AK9" t="inlineStr">
-        <is>
-          <t>cuspidata</t>
-        </is>
-      </c>
-      <c r="AN9" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="AO9" t="inlineStr">
-        <is>
-          <t>tree</t>
-        </is>
-      </c>
-      <c r="AP9" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AQ9" t="inlineStr">
-        <is>
-          <t>Nectandra cuspidata</t>
-        </is>
-      </c>
-      <c r="AR9" t="inlineStr">
-        <is>
-          <t>Nees &amp; Mart.</t>
-        </is>
-      </c>
-      <c r="AS9" t="inlineStr">
-        <is>
-          <t>Lauraceae</t>
-        </is>
-      </c>
-      <c r="AT9" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AU9" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AV9" t="inlineStr">
-        <is>
-          <t>Nectandra</t>
-        </is>
-      </c>
-      <c r="AW9" t="inlineStr">
-        <is>
-          <t>cuspidata</t>
-        </is>
-      </c>
-      <c r="AY9" t="inlineStr">
-        <is>
-          <t>NEC2</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>nectpu</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Damburneya umbrosa</t>
-        </is>
-      </c>
-      <c r="C10">
-        <v>86</v>
-      </c>
-      <c r="D10">
-        <v>2</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-      <c r="F10">
-        <v>1</v>
-      </c>
-      <c r="G10">
-        <v>14</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>bci50ha, bcimultiplots, bci10ha, P14, P11</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Laurales</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Lauraceae</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Damburneya</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>purpurea</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>(Ruiz &amp; Pav.) Trofimov</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Nectandra purpurea</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>R. Pérez 1872 (PMA, SCZ)</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>Freestanding</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>Damburneya purpurea</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>Damburneya purpurea</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>species</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>Damburneya purpurea</t>
-        </is>
-      </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>(Ruiz &amp; Pav.) Trofimov</t>
-        </is>
-      </c>
-      <c r="X10" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="Y10" t="inlineStr">
-        <is>
-          <t>Accepted</t>
-        </is>
-      </c>
-      <c r="Z10" t="inlineStr">
-        <is>
-          <t>3009192</t>
-        </is>
-      </c>
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>77158867-1</t>
-        </is>
-      </c>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC10" t="inlineStr">
-        <is>
-          <t>3009192</t>
-        </is>
-      </c>
-      <c r="AD10" t="inlineStr">
-        <is>
-          <t>77158867-1</t>
-        </is>
-      </c>
-      <c r="AE10" t="inlineStr">
-        <is>
-          <t>77158867-1</t>
-        </is>
-      </c>
-      <c r="AF10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AG10" t="inlineStr">
-        <is>
-          <t>Damburneya purpurea</t>
-        </is>
-      </c>
-      <c r="AH10" t="inlineStr">
-        <is>
-          <t>(Ruiz &amp; Pav.) Trofimov</t>
-        </is>
-      </c>
-      <c r="AI10" t="inlineStr">
-        <is>
-          <t>Lauraceae</t>
-        </is>
-      </c>
-      <c r="AJ10" t="inlineStr">
-        <is>
-          <t>Damburneya</t>
-        </is>
-      </c>
-      <c r="AK10" t="inlineStr">
-        <is>
-          <t>purpurea</t>
-        </is>
-      </c>
-      <c r="AN10" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="AO10" t="inlineStr">
-        <is>
-          <t>tree</t>
-        </is>
-      </c>
-      <c r="AP10" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AQ10" t="inlineStr">
-        <is>
-          <t>Damburneya purpurea</t>
-        </is>
-      </c>
-      <c r="AR10" t="inlineStr">
-        <is>
-          <t>(Ruiz &amp; Pav.) Trofimov</t>
-        </is>
-      </c>
-      <c r="AS10" t="inlineStr">
-        <is>
-          <t>Lauraceae</t>
-        </is>
-      </c>
-      <c r="AT10" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AU10" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AV10" t="inlineStr">
-        <is>
-          <t>Damburneya</t>
-        </is>
-      </c>
-      <c r="AW10" t="inlineStr">
-        <is>
-          <t>purpurea</t>
-        </is>
-      </c>
-      <c r="AY10" t="inlineStr">
-        <is>
-          <t>NECP</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>nects1</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Nectandra fuzzy</t>
-        </is>
-      </c>
-      <c r="C11">
-        <v>1</v>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11">
-        <v>0</v>
-      </c>
-      <c r="G11">
-        <v>0</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>bci50ha</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Lauraceae</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Nectandra</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>fuzzy</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>Nectandra sp.nov.1</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>Nectandra fuzzy</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>Nectandra fuzzy</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>genus</t>
-        </is>
-      </c>
-      <c r="AF11" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AQ11" t="inlineStr">
-        <is>
-          <t>Nectandra fuzzy</t>
-        </is>
-      </c>
-      <c r="AS11" t="inlineStr">
-        <is>
-          <t>Lauraceae</t>
-        </is>
-      </c>
-      <c r="AV11" t="inlineStr">
-        <is>
-          <t>Nectandra</t>
-        </is>
-      </c>
-      <c r="AW11" t="inlineStr">
-        <is>
-          <t>fuzzy</t>
-        </is>
-      </c>
-      <c r="AX11" t="inlineStr">
-        <is>
-          <t>Nectandra fuzzy</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>sapisp</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Sapium broadleaf</t>
-        </is>
-      </c>
-      <c r="C12">
-        <v>3</v>
-      </c>
-      <c r="D12">
-        <v>0</v>
-      </c>
-      <c r="E12">
-        <v>0</v>
-      </c>
-      <c r="F12">
-        <v>0</v>
-      </c>
-      <c r="G12">
-        <v>0</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>bci50ha</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Euphorbiaceae</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Sapium</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>broadleaf</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>Sapium broadleaf</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>Sapium broadleaf</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>genus</t>
-        </is>
-      </c>
-      <c r="AF12" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AQ12" t="inlineStr">
-        <is>
-          <t>Sapium broadleaf</t>
-        </is>
-      </c>
-      <c r="AS12" t="inlineStr">
-        <is>
-          <t>Euphorbiaceae</t>
-        </is>
-      </c>
-      <c r="AV12" t="inlineStr">
-        <is>
-          <t>Sapium</t>
-        </is>
-      </c>
-      <c r="AW12" t="inlineStr">
-        <is>
-          <t>broadleaf</t>
-        </is>
-      </c>
-      <c r="AX12" t="inlineStr">
-        <is>
-          <t>Sapium broadleaf</t>
-        </is>
-      </c>
-      <c r="AY12" t="inlineStr">
-        <is>
-          <t>SAPS</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>unonpa</t>
-        </is>
-      </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13">
-        <v>0</v>
-      </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
-      <c r="F13">
-        <v>0</v>
-      </c>
-      <c r="G13">
-        <v>1</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>bcimultiplots</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Magnoliales</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Annonaceae</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Unonopsis</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>panamensis</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>R.E. Fr.</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>R. Pérez 2303 (PMA, SCZ)</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>Freestanding</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>Unonopsis panamensis</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>Unonopsis panamensis</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>species</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>Unonopsis panamensis</t>
-        </is>
-      </c>
-      <c r="W13" t="inlineStr">
-        <is>
-          <t>R.E.Fr.</t>
-        </is>
-      </c>
-      <c r="X13" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="Y13" t="inlineStr">
-        <is>
-          <t>Accepted</t>
-        </is>
-      </c>
-      <c r="Z13" t="inlineStr">
-        <is>
-          <t>2447472</t>
-        </is>
-      </c>
-      <c r="AA13" t="inlineStr">
-        <is>
-          <t>259517-2</t>
-        </is>
-      </c>
-      <c r="AB13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC13" t="inlineStr">
-        <is>
-          <t>2447472</t>
-        </is>
-      </c>
-      <c r="AD13" t="inlineStr">
-        <is>
-          <t>259517-2</t>
-        </is>
-      </c>
-      <c r="AE13" t="inlineStr">
-        <is>
-          <t>259517-2</t>
-        </is>
-      </c>
-      <c r="AF13" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AG13" t="inlineStr">
-        <is>
-          <t>Unonopsis panamensis</t>
-        </is>
-      </c>
-      <c r="AH13" t="inlineStr">
-        <is>
-          <t>R.E.Fr.</t>
-        </is>
-      </c>
-      <c r="AI13" t="inlineStr">
-        <is>
-          <t>Annonaceae</t>
-        </is>
-      </c>
-      <c r="AJ13" t="inlineStr">
-        <is>
-          <t>Unonopsis</t>
-        </is>
-      </c>
-      <c r="AK13" t="inlineStr">
-        <is>
-          <t>panamensis</t>
-        </is>
-      </c>
-      <c r="AN13" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="AO13" t="inlineStr">
-        <is>
-          <t>tree</t>
-        </is>
-      </c>
-      <c r="AP13" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AQ13" t="inlineStr">
-        <is>
-          <t>Unonopsis panamensis</t>
-        </is>
-      </c>
-      <c r="AR13" t="inlineStr">
-        <is>
-          <t>R.E.Fr.</t>
-        </is>
-      </c>
-      <c r="AS13" t="inlineStr">
-        <is>
-          <t>Annonaceae</t>
-        </is>
-      </c>
-      <c r="AT13" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AU13" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AV13" t="inlineStr">
-        <is>
-          <t>Unonopsis</t>
-        </is>
-      </c>
-      <c r="AW13" t="inlineStr">
-        <is>
-          <t>panamensis</t>
-        </is>
-      </c>
-      <c r="AY13" t="inlineStr">
         <is>
           <t>UNO2</t>
         </is>

</xml_diff>